<commit_message>
MANUALES DE MIS PARTES A DOCUMENTAR
</commit_message>
<xml_diff>
--- a/Documentacion Sprint (01 - 11)/Sprint 11 documentacion/Sprint_11_Backlog_ICARO.xlsx
+++ b/Documentacion Sprint (01 - 11)/Sprint 11 documentacion/Sprint_11_Backlog_ICARO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\Sistema_Gestion_Integral_Constructora\Documentacion Sprint (01 - 11)\Sprint 11 documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772B7254-6D94-43AB-87F0-1F59C18271DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F15150-4C05-4AA9-BF55-97053D0A5C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30270" yWindow="1470" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Backlog 11" sheetId="4" r:id="rId1"/>
@@ -1025,107 +1025,107 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1134,41 +1134,6 @@
     <cellStyle name="Notas" xfId="1" builtinId="10"/>
   </cellStyles>
   <dxfs count="6">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -1260,6 +1225,41 @@
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1274,13 +1274,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3827E284-1C3B-4257-AEE7-2DAF0E64056F}" name="Tabla3" displayName="Tabla3" ref="A2:D14" totalsRowShown="0" headerRowDxfId="0" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3827E284-1C3B-4257-AEE7-2DAF0E64056F}" name="Tabla3" displayName="Tabla3" ref="A2:D14" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A2:D14" xr:uid="{3827E284-1C3B-4257-AEE7-2DAF0E64056F}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{27D72E59-B31B-4A27-A388-B1CFB7407A17}" name="Métrica" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{40490836-8515-4ED4-9303-CC2D488A9782}" name="Planificado" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{B86B6FFA-DFA0-4F58-97B7-E4F41070C797}" name="Realizado" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{98D1F4E8-4BBF-48C4-BE93-90278190BFC6}" name="Observación" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{27D72E59-B31B-4A27-A388-B1CFB7407A17}" name="Métrica" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{40490836-8515-4ED4-9303-CC2D488A9782}" name="Planificado" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{B86B6FFA-DFA0-4F58-97B7-E4F41070C797}" name="Realizado" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{98D1F4E8-4BBF-48C4-BE93-90278190BFC6}" name="Observación" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1585,407 +1585,402 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="12" t="s">
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
     </row>
     <row r="4" spans="1:12" ht="24">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="12" t="s">
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="H4" s="17">
+      <c r="H4" s="35">
         <v>46199</v>
       </c>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
     </row>
     <row r="5" spans="1:12" ht="132" customHeight="1">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="12" t="s">
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" spans="1:12" ht="24">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="12" t="s">
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-    </row>
-    <row r="7" spans="1:12" ht="30">
-      <c r="A7" s="19" t="s">
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="I7" s="20" t="s">
+      <c r="I7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="19" t="s">
+      <c r="J7" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="K7" s="19" t="s">
+      <c r="K7" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="8" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="174.75" customHeight="1">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="10">
         <v>5</v>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="10">
         <v>5</v>
       </c>
-      <c r="H8" s="21" t="s">
+      <c r="H8" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="I8" s="29" t="s">
+      <c r="I8" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="K8" s="21" t="s">
+      <c r="K8" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="L8" s="28" t="s">
+      <c r="L8" s="15" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="195">
-      <c r="A9" s="27" t="s">
+    <row r="9" spans="1:12" ht="165">
+      <c r="A9" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="10">
         <v>4</v>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="10">
         <v>4</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="I9" s="29" t="s">
+      <c r="I9" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="K9" s="21" t="s">
+      <c r="K9" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="L9" s="28" t="s">
+      <c r="L9" s="15" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="225">
-      <c r="A10" s="27" t="s">
+    <row r="10" spans="1:12" ht="180">
+      <c r="A10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="E10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="10">
         <v>6</v>
       </c>
-      <c r="G10" s="21">
+      <c r="G10" s="10">
         <v>6</v>
       </c>
-      <c r="H10" s="21" t="s">
+      <c r="H10" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="I10" s="29" t="s">
+      <c r="I10" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J10" s="21" t="s">
+      <c r="J10" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="K10" s="21" t="s">
+      <c r="K10" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="L10" s="21" t="s">
+      <c r="L10" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="135">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="E11" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="10">
         <v>5</v>
       </c>
-      <c r="G11" s="21">
+      <c r="G11" s="10">
         <v>5</v>
       </c>
-      <c r="H11" s="21" t="s">
+      <c r="H11" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="I11" s="29" t="s">
+      <c r="I11" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J11" s="21" t="s">
+      <c r="J11" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="K11" s="21" t="s">
+      <c r="K11" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="L11" s="21" t="s">
+      <c r="L11" s="10" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:12">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="25">
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="13">
         <v>20</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="13">
         <v>20</v>
       </c>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
     </row>
     <row r="14" spans="1:12">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
     </row>
     <row r="15" spans="1:12">
-      <c r="A15" s="30"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
+      <c r="A15" s="32"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
     </row>
     <row r="16" spans="1:12">
-      <c r="A16" s="30"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
+      <c r="A16" s="32"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
+      <c r="A17" s="32"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="30"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
+      <c r="A18" s="32"/>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="30"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
+      <c r="A19" s="32"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="30"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
+      <c r="A20" s="32"/>
+      <c r="B20" s="32"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="H5:L5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="H6:L6"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A14:G20"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -1993,6 +1988,11 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="H4:L4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="H5:L5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2011,14 +2011,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
@@ -2340,192 +2340,192 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="23" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="11">
         <v>20</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="11">
         <v>20</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="11" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="11">
         <v>0</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="11">
         <v>0</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="11" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="11">
         <v>4</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="11">
         <v>4</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="11" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="11">
         <v>4</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="11">
         <v>4</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="11" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="11">
         <v>4</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="11">
         <v>4</v>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="11">
         <v>0</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="11">
         <v>0</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="11" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="11">
         <v>0</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="11">
         <v>0</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="11" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="11">
         <v>20</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="11">
         <v>20</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="11" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="38">
+      <c r="B11" s="22">
         <v>1</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="22">
         <v>1</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="11" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="11">
         <v>14</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="11">
         <v>14</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="11" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="20.25" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="B13" s="38">
+      <c r="B13" s="22">
         <v>1</v>
       </c>
-      <c r="C13" s="38">
+      <c r="C13" s="22">
         <v>1</v>
       </c>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="11" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="17.25" customHeight="1">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="11">
         <v>268</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="11">
         <v>268</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="11" t="s">
         <v>189</v>
       </c>
     </row>
@@ -2550,185 +2550,185 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="39" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="17" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="19" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="21" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="19" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="21" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="19" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="21" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="21" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="19" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="21" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="34" t="s">
+      <c r="A13" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="C13" s="35" t="s">
+      <c r="C13" s="19" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="21" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="C15" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="21" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="19" t="s">
         <v>161</v>
       </c>
     </row>

</xml_diff>